<commit_message>
Simplify employee schedule entry in Excel template
Replace per-day time columns with Name, Role, Office, Working Days,
Start Time, End Time — one row per shift pattern. Includes day format
reference guide and common day range dropdown.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pto-app/PTO_Approval_Template.xlsx
+++ b/pto-app/PTO_Approval_Template.xlsx
@@ -20,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="HH:MM"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +91,25 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <color rgb="001A3A6B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009AA0B0"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005A6479"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -100,15 +118,14 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001A3A6B"/>
-      <sz val="16"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
+      <color rgb="001A3A6B"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -171,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,23 +213,33 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -220,17 +247,17 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -688,7 +715,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Go to the Employees sheet. Enter each staff member's name, role (Manager or Researcher), office, and typical working hours in EST for each day they work. Leave days blank if they don't work that day.</t>
+          <t>Go to the Employees sheet. Enter each staff member's name, role, office, working days, and shift hours in EST. Use a new row if someone has different hours on different days.</t>
         </is>
       </c>
     </row>
@@ -707,7 +734,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Go to the Coverage Rules sheet. Review the minimum staffing thresholds for each shift. Edit the blue values if your requirements change.</t>
+          <t>Go to the Coverage Rules sheet. Review the minimum staffing thresholds per shift. Edit the blue values if your requirements change.</t>
         </is>
       </c>
     </row>
@@ -726,7 +753,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Go to the PTO Requests sheet. Enter the employee's name, start/end dates, and request type.</t>
+          <t>Go to the PTO Requests sheet. Enter the employee, dates, and type.</t>
         </is>
       </c>
     </row>
@@ -745,7 +772,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Go to the Coverage Summary sheet. Enter the request's date range to see projected staffing levels. Check that each shift meets the minimums on the Coverage Rules sheet.</t>
+          <t>Go to the Coverage Summary sheet. Enter the request date range to review projected staffing levels against the minimums.</t>
         </is>
       </c>
     </row>
@@ -764,7 +791,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Return to PTO Requests and set the Status to Approved, Denied, or Pending based on the coverage check.</t>
+          <t>Return to PTO Requests and set the Status to Approved, Denied, or Pending.</t>
         </is>
       </c>
     </row>
@@ -776,14 +803,14 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Import Existing Absences</t>
+          <t>Import Existing</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>If importing from your absence system, paste dates into the PTO Requests sheet directly with Status = Approved.</t>
+          <t>For absences already on the calendar, enter them on the PTO Requests sheet with Status = Approved. You can paste multiple rows at once.</t>
         </is>
       </c>
     </row>
@@ -958,32 +985,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="2" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Employee Roster — Enter all staff with their typical working hours in EST. Leave time cells blank for days the employee does not work.</t>
+          <t>Enter each employee below with their shift. Use one row per shift pattern — add a second row for the same person if they have different hours on different days. All times in EST.</t>
         </is>
       </c>
     </row>
@@ -1005,431 +1026,453 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Mon
-Start</t>
+          <t>Working Days</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Mon
-End</t>
+          <t>Start Time
+(EST)</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Tue
-Start</t>
+          <t>End Time
+(EST)</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Tue
-End</t>
-        </is>
-      </c>
-      <c r="H2" s="8" t="inlineStr">
-        <is>
-          <t>Wed
-Start</t>
-        </is>
-      </c>
-      <c r="I2" s="8" t="inlineStr">
-        <is>
-          <t>Wed
-End</t>
-        </is>
-      </c>
-      <c r="J2" s="8" t="inlineStr">
-        <is>
-          <t>Thu
-Start</t>
-        </is>
-      </c>
-      <c r="K2" s="8" t="inlineStr">
-        <is>
-          <t>Thu
-End</t>
-        </is>
-      </c>
-      <c r="L2" s="8" t="inlineStr">
-        <is>
-          <t>Fri
-Start</t>
-        </is>
-      </c>
-      <c r="M2" s="8" t="inlineStr">
-        <is>
-          <t>Fri
-End</t>
-        </is>
-      </c>
-      <c r="N2" s="8" t="inlineStr">
-        <is>
-          <t>Sat
-Start</t>
-        </is>
-      </c>
-      <c r="O2" s="8" t="inlineStr">
-        <is>
-          <t>Sat
-End</t>
-        </is>
-      </c>
-      <c r="P2" s="8" t="inlineStr">
-        <is>
-          <t>Sun
-Start</t>
-        </is>
-      </c>
-      <c r="Q2" s="8" t="inlineStr">
-        <is>
-          <t>Sun
-End</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr"/>
-      <c r="B3" s="13" t="inlineStr">
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>Working Days — accepted formats</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>John Smith</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="J3" s="18" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="K3" s="19" t="inlineStr">
+        <is>
+          <t>Monday through Friday</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Sarah Chen</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Boston</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="G4" s="23" t="inlineStr"/>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>Mon-Thu</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="K4" s="19" t="inlineStr">
+        <is>
+          <t>Monday through Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>James Liu</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Overnight EST</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Tue-Sat</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="K5" s="19" t="inlineStr">
+        <is>
+          <t>Tuesday through Saturday</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>Emma Clarke</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr"/>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>Mon-Sun</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>Every day</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Mike Torres</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr"/>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Sat-Sun</t>
+        </is>
+      </c>
+      <c r="J7" s="18" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>Weekends only</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Priya Sharma</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="L3" s="13" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="M3" s="13" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="N3" s="14" t="inlineStr"/>
-      <c r="O3" s="14" t="inlineStr"/>
-      <c r="P3" s="14" t="inlineStr"/>
-      <c r="Q3" s="14" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="15" t="inlineStr"/>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="G8" s="23" t="inlineStr"/>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>Mon, Wed, Fri</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="K8" s="19" t="inlineStr">
+        <is>
+          <t>Specific days</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Priya Sharma</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Researcher</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Sat-Sun</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Weekend on-call</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>Mon only</t>
+        </is>
+      </c>
+      <c r="J9" s="18" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>Single day</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>David Park</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Researcher</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>New York</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="G4" s="16" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="H4" s="16" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="I4" s="16" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="J4" s="16" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="L4" s="16" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="M4" s="16" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="N4" s="17" t="inlineStr"/>
-      <c r="O4" s="17" t="inlineStr"/>
-      <c r="P4" s="17" t="inlineStr"/>
-      <c r="Q4" s="17" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr"/>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Researcher</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>Hong Kong</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Tue-Sat</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Lisa Wang</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Mon-Fri</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>08:00</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="K5" s="13" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="L5" s="13" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="M5" s="13" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="N5" s="14" t="inlineStr"/>
-      <c r="O5" s="14" t="inlineStr"/>
-      <c r="P5" s="14" t="inlineStr"/>
-      <c r="Q5" s="14" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr"/>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Researcher</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="H6" s="16" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="I6" s="16" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="J6" s="16" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="K6" s="16" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="L6" s="16" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="M6" s="16" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="N6" s="17" t="inlineStr"/>
-      <c r="O6" s="17" t="inlineStr"/>
-      <c r="P6" s="17" t="inlineStr"/>
-      <c r="Q6" s="17" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr"/>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Los Angeles</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="H7" s="13" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="M7" s="13" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="N7" s="14" t="inlineStr"/>
-      <c r="O7" s="14" t="inlineStr"/>
-      <c r="P7" s="14" t="inlineStr"/>
-      <c r="Q7" s="14" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:S1"/>
+  <mergeCells count="2">
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="B3:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Manager,Researcher"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D3:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Mon-Fri,Mon-Thu,Tue-Sat,Wed-Sun,Mon-Sat,Mon-Sun,Sat-Sun,Mon only,Tue only,Wed only,Thu only,Fri only,Sat only,Sun only"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1462,7 +1505,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>PTO Requests — Enter each request below. Use the Coverage Summary sheet to verify coverage before setting Status.</t>
+          <t>Enter PTO requests below. Use Coverage Summary to verify coverage before approving. For imported absences set Status = Approved.</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1574,12 @@
           <t>PTO-001</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
-        <is>
-          <t>Jane Smith</t>
-        </is>
-      </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>John Smith</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Researcher</t>
         </is>
@@ -1556,7 +1599,7 @@
           <t>Vacation</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr"/>
+      <c r="G3" s="24" t="inlineStr"/>
       <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1582,12 +1625,12 @@
           <t>PTO-002</t>
         </is>
       </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>John Doe</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Sarah Chen</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
@@ -1607,7 +1650,7 @@
           <t>Sick</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr"/>
+      <c r="G4" s="25" t="inlineStr"/>
       <c r="H4" s="10" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1633,12 +1676,12 @@
           <t>PTO-003</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Alex Johnson</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Emma Clarke</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>Researcher</t>
         </is>
@@ -1658,7 +1701,7 @@
           <t>Vacation</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Pre-planned</t>
         </is>
@@ -1742,7 +1785,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Coverage Rules</t>
         </is>
@@ -1751,7 +1794,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Edit the blue values to adjust staffing thresholds. These are referenced by the Coverage Summary sheet.</t>
+          <t>Edit the blue values to adjust staffing thresholds. Values here flow into the Coverage Summary sheet.</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1808,7 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Managers are only counted Mon–Fri. The Daytime shift requires at least 2 managers online.</t>
+          <t>Shift windows are defined in EST. Managers are only counted Mon–Fri.</t>
         </is>
       </c>
     </row>
@@ -1802,78 +1845,78 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Morning</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>Midnight – 9am</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>Overnight coverage — thin by design</t>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>Overnight — thin by design</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Daytime</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>9am – 5pm</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="15" t="inlineStr">
-        <is>
-          <t>Core business hours — manager presence required</t>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>Core hours — manager presence required</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Evening</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>5pm – Midnight</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>US West Coast wind-down</t>
         </is>
@@ -1882,7 +1925,7 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Shift name reference: Morning = rows 7, Daytime = row 8, Evening = row 9</t>
+          <t>Row reference: Morning = row 7, Daytime = row 8, Evening = row 9 (used in Coverage Summary formulas)</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1939,7 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Maximum number of employees who may have approved PTO on a weekend day. No manager coverage is required on weekends.</t>
+          <t>Maximum number of employees who may be approved off on a weekend day. No manager coverage required on weekends.</t>
         </is>
       </c>
     </row>
@@ -1918,30 +1961,30 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>Only 1 employee may be approved off on any given Saturday</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B17" s="22" t="n">
+      <c r="B17" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="28" t="inlineStr">
         <is>
           <t>Only 1 employee may be approved off on any given Sunday</t>
         </is>
@@ -1976,11 +2019,11 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Coverage Summary</t>
         </is>
@@ -1994,78 +2037,71 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Start Date:</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="29" t="inlineStr">
         <is>
           <t>End Date:</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="30" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="G5" s="25" t="inlineStr">
-        <is>
-          <t>↑ Yellow cells are editable</t>
+      <c r="G5" s="31" t="inlineStr">
+        <is>
+          <t>← Yellow cells are editable</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>How to use this sheet:</t>
+          <t>How to use:</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>1. Enter your date range above (B5 and E5)</t>
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>1. Enter the PTO request's date range in B5 and E5</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>2. For each day in the range, manually count staff scheduled vs. approved off using the Employees and PTO Requests sheets</t>
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>2. For each day, count staff scheduled (from Employees sheet) minus those with approved PTO (from PTO Requests sheet)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>3. Compare totals against the minimums on the Coverage Rules sheet</t>
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>3. Compare against minimums below — mark OK if met, REVIEW if not</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>4. Mark the Status column: OK (meets minimums) or REVIEW (below minimums)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>5. Return to PTO Requests to approve or deny the request</t>
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>4. Return to PTO Requests to set the final Status</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Quick Reference — Minimum Staffing per Shift (from Coverage Rules sheet)</t>
+          <t>Minimum Staffing Reference (live from Coverage Rules sheet)</t>
         </is>
       </c>
     </row>
@@ -2097,73 +2133,73 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>Morning</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Midnight – 9am</t>
         </is>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="27">
         <f>'Coverage Rules'!C7</f>
         <v/>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="27">
         <f>'Coverage Rules'!D7</f>
         <v/>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="27">
         <f>'Coverage Rules'!E7</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>Daytime</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>9am – 5pm</t>
         </is>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="28">
         <f>'Coverage Rules'!C8</f>
         <v/>
       </c>
-      <c r="D17" s="17">
+      <c r="D17" s="28">
         <f>'Coverage Rules'!D8</f>
         <v/>
       </c>
-      <c r="E17" s="17">
+      <c r="E17" s="28">
         <f>'Coverage Rules'!E8</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>Evening</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>5pm – Midnight</t>
         </is>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="27">
         <f>'Coverage Rules'!C9</f>
         <v/>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="27">
         <f>'Coverage Rules'!D9</f>
         <v/>
       </c>
-      <c r="E18" s="14">
+      <c r="E18" s="27">
         <f>'Coverage Rules'!E9</f>
         <v/>
       </c>
@@ -2171,7 +2207,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Daily Coverage Tracker — Fill in manually for the requested date range</t>
+          <t>Daily Coverage Tracker</t>
         </is>
       </c>
     </row>
@@ -2229,235 +2265,234 @@
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr"/>
-      <c r="F23" s="14" t="inlineStr"/>
-      <c r="G23" s="13" t="n">
+      <c r="E23" s="27" t="inlineStr"/>
+      <c r="F23" s="27" t="inlineStr"/>
+      <c r="G23" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="13" t="inlineStr">
+      <c r="H23" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I23" s="12" t="inlineStr"/>
+      <c r="I23" s="16" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="28" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
       </c>
-      <c r="C24" s="17" t="inlineStr"/>
-      <c r="D24" s="17" t="inlineStr"/>
-      <c r="E24" s="16" t="n">
+      <c r="C24" s="28" t="inlineStr"/>
+      <c r="D24" s="28" t="inlineStr"/>
+      <c r="E24" s="21" t="n">
         <v>32</v>
       </c>
-      <c r="F24" s="16" t="inlineStr">
+      <c r="F24" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G24" s="16" t="n">
+      <c r="G24" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="H24" s="16" t="inlineStr">
+      <c r="H24" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I24" s="15" t="inlineStr"/>
+      <c r="I24" s="23" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr"/>
-      <c r="D25" s="14" t="inlineStr"/>
-      <c r="E25" s="13" t="n">
+      <c r="C25" s="27" t="inlineStr"/>
+      <c r="D25" s="27" t="inlineStr"/>
+      <c r="E25" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G25" s="13" t="n">
+      <c r="G25" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="H25" s="13" t="inlineStr">
+      <c r="H25" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I25" s="12" t="inlineStr"/>
+      <c r="I25" s="16" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="28" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C26" s="17" t="inlineStr"/>
-      <c r="D26" s="17" t="inlineStr"/>
-      <c r="E26" s="16" t="n">
+      <c r="C26" s="28" t="inlineStr"/>
+      <c r="D26" s="28" t="inlineStr"/>
+      <c r="E26" s="21" t="n">
+        <v>29</v>
+      </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="G26" s="21" t="n">
+        <v>19</v>
+      </c>
+      <c r="H26" s="21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" s="23" t="inlineStr">
+        <is>
+          <t>John Smith off — check daytime min</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="inlineStr"/>
+      <c r="D27" s="27" t="inlineStr"/>
+      <c r="E27" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="inlineStr"/>
+      <c r="D28" s="28" t="inlineStr"/>
+      <c r="E28" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>REVIEW</t>
-        </is>
-      </c>
-      <c r="G26" s="16" t="n">
-        <v>19</v>
-      </c>
-      <c r="H26" s="16" t="inlineStr">
+      <c r="F28" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I26" s="15" t="inlineStr">
-        <is>
-          <t>Check daytime — 2 approved off</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr"/>
-      <c r="D27" s="14" t="inlineStr"/>
-      <c r="E27" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="G28" s="21" t="n">
+        <v>17</v>
+      </c>
+      <c r="H28" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G27" s="13" t="n">
-        <v>22</v>
-      </c>
-      <c r="H27" s="13" t="inlineStr">
+      <c r="I28" s="23" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I27" s="12" t="inlineStr"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="inlineStr"/>
-      <c r="D28" s="17" t="inlineStr"/>
-      <c r="E28" s="16" t="n">
-        <v>29</v>
-      </c>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr"/>
+      <c r="F29" s="27" t="inlineStr"/>
+      <c r="G29" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G28" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="H28" s="16" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" s="15" t="inlineStr"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>Saturday</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr"/>
-      <c r="F29" s="14" t="inlineStr"/>
-      <c r="G29" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" s="12" t="inlineStr"/>
+      <c r="I29" s="16" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="7">
     <mergeCell ref="A11:I11"/>
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="A8:I8"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A12:I12"/>
     <mergeCell ref="A21:I21"/>
   </mergeCells>
   <conditionalFormatting sqref="D23:D200">

</xml_diff>

<commit_message>
Split Evening shift into EST and PST sub-windows
Evening (EST): 5pm-9pm EST, min 1 staff (1pm-9pm EST shift)
Evening (PST): 5pm-midnight EST, min 2 staff (1pm-9pm PST shift)
Coverage Summary reference table updated to match.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pto-app/PTO_Approval_Template.xlsx
+++ b/pto-app/PTO_Approval_Template.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="HH:MM"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -133,6 +133,12 @@
       <color rgb="000000FF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -188,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -260,6 +266,12 @@
     <xf numFmtId="165" fontId="18" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -667,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F31"/>
+  <dimension ref="A2:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -893,73 +905,94 @@
     <row r="29">
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>Evening (EST)</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>5pm – Midnight</t>
+          <t>5pm – 9pm EST</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
+          <t>Evening (PST)</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>5pm – Midnight EST</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="10" t="inlineStr">
+        <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>Any</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>Max 1 off</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="9" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Any</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>Max 1 off</t>
         </is>
@@ -1773,7 +1806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1845,157 +1878,186 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Morning</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>Midnight – 9am</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="n">
+          <t>Midnight – 9am EST</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Overnight floor — HK team + early starters</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>Daytime</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>9am – 5pm EST</t>
+        </is>
+      </c>
+      <c r="C8" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Core hours — 2 managers required</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Evening (EST)</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>5pm – 9pm EST</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="27" t="inlineStr">
-        <is>
-          <t>Overnight — thin by design</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="23" t="inlineStr">
-        <is>
-          <t>Daytime</t>
-        </is>
-      </c>
-      <c r="B8" s="28" t="inlineStr">
-        <is>
-          <t>9am – 5pm</t>
-        </is>
-      </c>
-      <c r="C8" s="21" t="n">
+      <c r="E9" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>At least 1 person on 1pm–9pm EST shift</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>Evening (PST)</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>5pm – Midnight EST</t>
+        </is>
+      </c>
+      <c r="C10" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="E8" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="F8" s="28" t="inlineStr">
-        <is>
-          <t>Core hours — manager presence required</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Evening</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="inlineStr">
-        <is>
-          <t>5pm – Midnight</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F9" s="27" t="inlineStr">
-        <is>
-          <t>US West Coast wind-down</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Row reference: Morning = row 7, Daytime = row 8, Evening = row 9 (used in Coverage Summary formulas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="E10" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>At least 2 people on 1pm–9pm PST (4pm–midnight EST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Row reference: Morning = row 7, Daytime = row 8, Evening (EST) = row 9, Evening (PST) = row 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>B. Weekend Rules</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Maximum number of employees who may be approved off on a weekend day. No manager coverage required on weekends.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Max People Off</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B17" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>Only 1 employee may be approved off on any given Saturday</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="23" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B18" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="28" t="inlineStr">
+      <c r="C18" s="28" t="inlineStr">
         <is>
           <t>Only 1 employee may be approved off on any given Sunday</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2008,7 +2070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2140,7 +2202,7 @@
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Midnight – 9am</t>
+          <t>Midnight – 9am EST</t>
         </is>
       </c>
       <c r="C16" s="27">
@@ -2164,7 +2226,7 @@
       </c>
       <c r="B17" s="28" t="inlineStr">
         <is>
-          <t>9am – 5pm</t>
+          <t>9am – 5pm EST</t>
         </is>
       </c>
       <c r="C17" s="28">
@@ -2183,12 +2245,12 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>Evening (EST)</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>5pm – Midnight</t>
+          <t>5pm – 9pm EST</t>
         </is>
       </c>
       <c r="C18" s="27">
@@ -2204,286 +2266,312 @@
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>Evening (PST)</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>5pm – Midnight EST</t>
+        </is>
+      </c>
+      <c r="C19" s="28">
+        <f>'Coverage Rules'!C10</f>
+        <v/>
+      </c>
+      <c r="D19" s="28">
+        <f>'Coverage Rules'!D10</f>
+        <v/>
+      </c>
+      <c r="E19" s="28">
+        <f>'Coverage Rules'!E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Daily Coverage Tracker</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Morning
 Staff</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Morning
 Status</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Daytime
 Staff</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Daytime
 Status</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>Evening
 Staff</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>Evening
 Status</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
+      <c r="C24" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E23" s="27" t="inlineStr"/>
-      <c r="F23" s="27" t="inlineStr"/>
-      <c r="G23" s="14" t="n">
+      <c r="E24" s="27" t="inlineStr"/>
+      <c r="F24" s="27" t="inlineStr"/>
+      <c r="G24" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="H24" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I23" s="16" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="I24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="B24" s="28" t="inlineStr">
+      <c r="B25" s="28" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
       </c>
-      <c r="C24" s="28" t="inlineStr"/>
-      <c r="D24" s="28" t="inlineStr"/>
-      <c r="E24" s="21" t="n">
+      <c r="C25" s="28" t="inlineStr"/>
+      <c r="D25" s="28" t="inlineStr"/>
+      <c r="E25" s="21" t="n">
         <v>32</v>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F25" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G24" s="21" t="n">
+      <c r="G25" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="H24" s="21" t="inlineStr">
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I24" s="23" t="inlineStr"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="I25" s="23" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="B25" s="27" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="C25" s="27" t="inlineStr"/>
-      <c r="D25" s="27" t="inlineStr"/>
-      <c r="E25" s="14" t="n">
+      <c r="C26" s="27" t="inlineStr"/>
+      <c r="D26" s="27" t="inlineStr"/>
+      <c r="E26" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G25" s="14" t="n">
+      <c r="G26" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="H25" s="14" t="inlineStr">
+      <c r="H26" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I25" s="16" t="inlineStr"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="B26" s="28" t="inlineStr">
+      <c r="B27" s="28" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="C26" s="28" t="inlineStr"/>
-      <c r="D26" s="28" t="inlineStr"/>
-      <c r="E26" s="21" t="n">
+      <c r="C27" s="28" t="inlineStr"/>
+      <c r="D27" s="28" t="inlineStr"/>
+      <c r="E27" s="21" t="n">
         <v>29</v>
       </c>
-      <c r="F26" s="21" t="inlineStr">
+      <c r="F27" s="21" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="G26" s="21" t="n">
+      <c r="G27" s="21" t="n">
         <v>19</v>
       </c>
-      <c r="H26" s="21" t="inlineStr">
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I26" s="23" t="inlineStr">
+      <c r="I27" s="23" t="inlineStr">
         <is>
           <t>John Smith off — check daytime min</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="B27" s="27" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C27" s="27" t="inlineStr"/>
-      <c r="D27" s="27" t="inlineStr"/>
-      <c r="E27" s="14" t="n">
+      <c r="C28" s="27" t="inlineStr"/>
+      <c r="D28" s="27" t="inlineStr"/>
+      <c r="E28" s="14" t="n">
         <v>33</v>
       </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
+      <c r="G28" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="H27" s="14" t="inlineStr">
+      <c r="H28" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I27" s="16" t="inlineStr"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="B28" s="28" t="inlineStr">
+      <c r="B29" s="28" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
       </c>
-      <c r="C28" s="28" t="inlineStr"/>
-      <c r="D28" s="28" t="inlineStr"/>
-      <c r="E28" s="21" t="n">
+      <c r="C29" s="28" t="inlineStr"/>
+      <c r="D29" s="28" t="inlineStr"/>
+      <c r="E29" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="F29" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="G28" s="21" t="n">
+      <c r="G29" s="21" t="n">
         <v>17</v>
       </c>
-      <c r="H28" s="21" t="inlineStr">
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I28" s="23" t="inlineStr"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="I29" s="23" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
+      <c r="C30" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E29" s="27" t="inlineStr"/>
-      <c r="F29" s="27" t="inlineStr"/>
-      <c r="G29" s="14" t="n">
+      <c r="E30" s="27" t="inlineStr"/>
+      <c r="F30" s="27" t="inlineStr"/>
+      <c r="G30" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="14" t="inlineStr">
+      <c r="H30" s="14" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I29" s="16" t="inlineStr"/>
+      <c r="I30" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Add Early Morning coverage group rule
New Coverage Group column in Employees sheet to tag staff by group.
Section C in Coverage Rules defines group rules: Early Morning group
(3 staff, 5am-3:30pm EST) allows max 2 out at once, min 1 present.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pto-app/PTO_Approval_Template.xlsx
+++ b/pto-app/PTO_Approval_Template.xlsx
@@ -194,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -272,6 +272,8 @@
     <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F32"/>
+  <dimension ref="B2:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1018,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1028,7 +1030,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="2" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="4" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -1037,7 +1039,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Enter each employee below with their shift. Use one row per shift pattern — add a second row for the same person if they have different hours on different days. All times in EST.</t>
+          <t>Enter each employee below with their shift. Use one row per shift pattern. If an employee belongs to a coverage group (e.g. Early Morning), enter the group name in the Coverage Group column. All times in EST.</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1081,13 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Coverage
+Group</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>Working Days — accepted formats</t>
         </is>
@@ -1117,17 +1125,18 @@
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr"/>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="H3" s="35" t="n"/>
+      <c r="J3" s="17" t="inlineStr">
         <is>
           <t>Mon-Fri</t>
         </is>
       </c>
-      <c r="J3" s="18" t="inlineStr">
+      <c r="K3" s="18" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="K3" s="19" t="inlineStr">
+      <c r="L3" s="19" t="inlineStr">
         <is>
           <t>Monday through Friday</t>
         </is>
@@ -1165,17 +1174,18 @@
         </is>
       </c>
       <c r="G4" s="23" t="inlineStr"/>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="H4" s="36" t="n"/>
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>Mon-Thu</t>
         </is>
       </c>
-      <c r="J4" s="18" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="K4" s="19" t="inlineStr">
+      <c r="L4" s="19" t="inlineStr">
         <is>
           <t>Monday through Thursday</t>
         </is>
@@ -1217,17 +1227,18 @@
           <t>Overnight EST</t>
         </is>
       </c>
-      <c r="I5" s="17" t="inlineStr">
+      <c r="H5" s="35" t="n"/>
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>Tue-Sat</t>
         </is>
       </c>
-      <c r="J5" s="18" t="inlineStr">
+      <c r="K5" s="18" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="K5" s="19" t="inlineStr">
+      <c r="L5" s="19" t="inlineStr">
         <is>
           <t>Tuesday through Saturday</t>
         </is>
@@ -1265,17 +1276,18 @@
         </is>
       </c>
       <c r="G6" s="23" t="inlineStr"/>
-      <c r="I6" s="17" t="inlineStr">
+      <c r="H6" s="36" t="n"/>
+      <c r="J6" s="17" t="inlineStr">
         <is>
           <t>Mon-Sun</t>
         </is>
       </c>
-      <c r="J6" s="18" t="inlineStr">
+      <c r="K6" s="18" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="K6" s="19" t="inlineStr">
+      <c r="L6" s="19" t="inlineStr">
         <is>
           <t>Every day</t>
         </is>
@@ -1313,17 +1325,18 @@
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr"/>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="H7" s="35" t="n"/>
+      <c r="J7" s="17" t="inlineStr">
         <is>
           <t>Sat-Sun</t>
         </is>
       </c>
-      <c r="J7" s="18" t="inlineStr">
+      <c r="K7" s="18" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="K7" s="19" t="inlineStr">
+      <c r="L7" s="19" t="inlineStr">
         <is>
           <t>Weekends only</t>
         </is>
@@ -1361,17 +1374,18 @@
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr"/>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="H8" s="36" t="n"/>
+      <c r="J8" s="17" t="inlineStr">
         <is>
           <t>Mon, Wed, Fri</t>
         </is>
       </c>
-      <c r="J8" s="18" t="inlineStr">
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="K8" s="19" t="inlineStr">
+      <c r="L8" s="19" t="inlineStr">
         <is>
           <t>Specific days</t>
         </is>
@@ -1413,17 +1427,18 @@
           <t>Weekend on-call</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
+      <c r="H9" s="35" t="n"/>
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>Mon only</t>
         </is>
       </c>
-      <c r="J9" s="18" t="inlineStr">
+      <c r="K9" s="18" t="inlineStr">
         <is>
           <t>→</t>
         </is>
       </c>
-      <c r="K9" s="19" t="inlineStr">
+      <c r="L9" s="19" t="inlineStr">
         <is>
           <t>Single day</t>
         </is>
@@ -1461,6 +1476,7 @@
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr"/>
+      <c r="H10" s="36" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
@@ -1494,6 +1510,31 @@
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr"/>
+      <c r="H11" s="35" t="n"/>
+    </row>
+    <row r="12">
+      <c r="H12" s="36" t="n"/>
+    </row>
+    <row r="13">
+      <c r="H13" s="35" t="n"/>
+    </row>
+    <row r="14">
+      <c r="H14" s="36" t="n"/>
+    </row>
+    <row r="15">
+      <c r="H15" s="35" t="n"/>
+    </row>
+    <row r="16">
+      <c r="H16" s="36" t="n"/>
+    </row>
+    <row r="17">
+      <c r="H17" s="35" t="n"/>
+    </row>
+    <row r="18">
+      <c r="H18" s="36" t="n"/>
+    </row>
+    <row r="19">
+      <c r="H19" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1806,7 +1847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1989,7 +2030,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
@@ -2051,13 +2091,94 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>C. Coverage Group Rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>These rules apply to named groups of employees tagged in the Coverage Group column of the Employees sheet. Unlike shift minimums, these rules restrict how many people from a specific group can be out simultaneously.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Group Name</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Hours (EST)</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Group Size</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Max Out at Once</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Min Present</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Early Morning</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>5am – 3:30pm EST</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>1 person at 5am–1pm, 1 at 7am–3pm, 1 at 7:30am–3:30pm. At least 1 must be present — max 2 out at a time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>How to use: When reviewing a PTO request, check how many other Early Morning group members already have approved time off on those dates. If 2 are already approved, deny the request or ask for coverage.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A26:F26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2290,7 +2411,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21"/>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="5" t="inlineStr">

</xml_diff>